<commit_message>
feat: 3.5k OAD tab, 1k tab, nav deep dive links, rolling stats fixes
- Add oad_game_theory_tab.py (3.5k OAD tab) with Miami Championship
- Add oad_solo_tab.py (1k OAD tab) with full 2026 schedule
- Add click-to-deep-dive nav on player photos/names throughout app
- Fix rolling stats to use all tours; NaN sub-stats default to 0
- Fix Euro player stat bar direction bug in sg_production_tab
- Add Alex Fitzpatrick to All_players
- Add Truist Championship approach bucket values
- Replace em dashes with hyphens across all tab scripts
- Gap to #7 (1k) and gap to #20 (3.5k)
- Add Miami Championship to schedule and OAD events

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/in Use/OAD_2026_Schedule.xlsx
+++ b/Data/in Use/OAD_2026_Schedule.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA30"/>
+  <dimension ref="A1:AA34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,323 +571,137 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46058</v>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
+        <v>46037</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>WM Phoenix Open</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>9600000</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1728000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>9600000</v>
-      </c>
+          <t>Sony Open in Hawaii</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>1728000</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>TPC Scottsdale</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>510</v>
-      </c>
+        <v>991900</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Thomas Detry</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://res.cloudinary.com/pgatour-prod/d_tournaments:logos:R000.png/tournaments/logos/R003.png</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
-        <v>71</v>
-      </c>
-      <c r="O2" t="n">
-        <v>7261</v>
-      </c>
-      <c r="P2" t="n">
-        <v>74.7</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>142</v>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Bermuda</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Bermuda</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Mix</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Scottsdale, AZ</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>60</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Thomas Detry</t>
-        </is>
-      </c>
-      <c r="X2" t="n">
-        <v>-25</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>-8</v>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>TPC Scottsdale, Scottsdale AZ</t>
-        </is>
-      </c>
-      <c r="AA2" t="n">
-        <v>65</v>
-      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
+        <v>46044</v>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AT&amp;T Pebble Beach Pro-Am</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3600000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>20000000</v>
-      </c>
+          <t>The American Express</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>3600000</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Pebble Beach</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>5</v>
-      </c>
+        <v>616400</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Rory McIlroy</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>https://res.cloudinary.com/pgatour-prod/d_tournaments:logos:R000.png/tournaments/logos/R005.png</t>
-        </is>
-      </c>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
-        <v>72</v>
-      </c>
-      <c r="O3" t="n">
-        <v>7075</v>
-      </c>
-      <c r="P3" t="n">
-        <v>75.90000000000001</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>148</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Poa annua</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Rye</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Ryegrass</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Pebble Beach, CA</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>62</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>David Duval</t>
-        </is>
-      </c>
-      <c r="X3" t="n">
-        <v>-19</v>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>No Cut</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>Pebble Beach, CA</t>
-        </is>
-      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46072</v>
-      </c>
-      <c r="B4" t="n">
-        <v>7</v>
-      </c>
+        <v>46051</v>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The Genesis Invitational</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="E4" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>20000000</v>
-      </c>
+          <t>Farmers Insurance Open</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Riviera Country Club</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>500</v>
-      </c>
+        <v>1728000</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Ludvig Aberg</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r007?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
-        <v>71</v>
-      </c>
-      <c r="O4" t="n">
-        <v>7383</v>
-      </c>
-      <c r="P4" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>135</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Poa annua</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Kikuyu</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Ryegrass</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Pacific Palisades, CA</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>62</v>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>Multiple players</t>
-        </is>
-      </c>
-      <c r="X4" t="n">
-        <v>-14</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>-2</v>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>Riviera Country Club, Pacific Palisades CA</t>
-        </is>
-      </c>
-      <c r="AA4" t="n">
-        <v>50</v>
-      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46079</v>
+        <v>46058</v>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cognizant Classic</t>
+          <t>WM Phoenix Open</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -904,11 +718,11 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PGA National</t>
+          <t>TPC Scottsdale</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>928</v>
+        <v>510</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -917,26 +731,26 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Joe Highsmith</t>
+          <t>Thomas Detry</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r010?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/d_tournaments:logos:R000.png/tournaments/logos/R003.png</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O5" t="n">
-        <v>7045</v>
+        <v>7261</v>
       </c>
       <c r="P5" t="n">
-        <v>75.3</v>
+        <v>74.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -950,31 +764,31 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Mix</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Palm Beach Gardens, FL</t>
+          <t>Scottsdale, AZ</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Thomas Detry</t>
         </is>
       </c>
       <c r="X5" t="n">
-        <v>-12</v>
+        <v>-25</v>
       </c>
       <c r="Y5" t="n">
-        <v>-1</v>
+        <v>-8</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>PGA National, Palm Beach Gardens FL</t>
+          <t>TPC Scottsdale, Scottsdale AZ</t>
         </is>
       </c>
       <c r="AA5" t="n">
@@ -983,35 +797,35 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46086</v>
+        <v>46065</v>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Arnold Palmer Invitational presented by Mastercard</t>
+          <t>AT&amp;T Pebble Beach Pro-Am</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>20000000</v>
       </c>
       <c r="E6" t="n">
-        <v>4000000</v>
+        <v>3600000</v>
       </c>
       <c r="F6" t="n">
         <v>20000000</v>
       </c>
       <c r="G6" t="n">
-        <v>4000000</v>
+        <v>3600000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Bay Hill</t>
+          <t>Pebble Beach</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1020,12 +834,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Russel Henley</t>
+          <t>Rory McIlroy</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r009?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/d_tournaments:logos:R000.png/tournaments/logos/R005.png</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1033,88 +847,88 @@
         <v>72</v>
       </c>
       <c r="O6" t="n">
-        <v>7381</v>
+        <v>7075</v>
       </c>
       <c r="P6" t="n">
-        <v>75.2</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="Q6" t="n">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Poa annua</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Rye</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Ryegrass</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>Pebble Beach, CA</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Ernie Els</t>
+          <t>David Duval</t>
         </is>
       </c>
       <c r="X6" t="n">
-        <v>-16</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>-3</v>
+        <v>-19</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>No Cut</t>
+        </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>Bay Hill Club, Orlando FL</t>
-        </is>
-      </c>
-      <c r="AA6" t="n">
-        <v>50</v>
-      </c>
+          <t>Pebble Beach, CA</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46093</v>
+        <v>46072</v>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>THE PLAYERS Championship</t>
+          <t>The Genesis Invitational</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>25000000</v>
+        <v>20000000</v>
       </c>
       <c r="E7" t="n">
-        <v>4500000</v>
+        <v>4000000</v>
       </c>
       <c r="F7" t="n">
-        <v>27777777.77</v>
+        <v>20000000</v>
       </c>
       <c r="G7" t="n">
-        <v>5000000</v>
+        <v>4000000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TPC Sawgrass</t>
+          <t>Riviera Country Club</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>11</v>
+        <v>500</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1123,57 +937,53 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Rory McIlroy</t>
+          <t>Ludvig Aberg</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r011?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>https://www.theplayers.com/news/2026/03/09/media_1a0195f4b8db5ca190f4d05315255fc352cf9c37d.jpg?width=2000&amp;format=webply&amp;optimize=medium</t>
-        </is>
-      </c>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r007?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O7" t="n">
-        <v>7245</v>
+        <v>7383</v>
       </c>
       <c r="P7" t="n">
-        <v>76.40000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="Q7" t="n">
-        <v>155</v>
+        <v>135</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Poa annua</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Kikuyu</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Ryegrass</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Ponte Vedra Beach, FL</t>
+          <t>Pacific Palisades, CA</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Fred Couples / Greg Norman</t>
+          <t>Multiple players</t>
         </is>
       </c>
       <c r="X7" t="n">
@@ -1184,44 +994,44 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>TPC Sawgrass, Ponte Vedra Beach FL</t>
+          <t>Riviera Country Club, Pacific Palisades CA</t>
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46100</v>
+        <v>46079</v>
       </c>
       <c r="B8" t="n">
-        <v>475</v>
+        <v>10</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Valspar Championship</t>
+          <t>Cognizant Classic in The Palm Beaches</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9100000</v>
+        <v>9600000</v>
       </c>
       <c r="E8" t="n">
-        <v>1638000</v>
+        <v>1728000</v>
       </c>
       <c r="F8" t="n">
-        <v>9100000</v>
+        <v>9600000</v>
       </c>
       <c r="G8" t="n">
-        <v>1638000</v>
+        <v>726400</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Innisbrook Resort</t>
+          <t>PGA National</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>665</v>
+        <v>928</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1230,26 +1040,26 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Viktor Hovland</t>
+          <t>Joe Highsmith</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r475?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r010?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O8" t="n">
-        <v>7340</v>
+        <v>7045</v>
       </c>
       <c r="P8" t="n">
-        <v>75.59999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1268,11 +1078,11 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Palm Harbor, FL</t>
+          <t>Palm Beach Gardens, FL</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1280,14 +1090,14 @@
         </is>
       </c>
       <c r="X8" t="n">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="Y8" t="n">
         <v>-1</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Innisbrook Resort, Palm Harbor FL</t>
+          <t>PGA National, Palm Beach Gardens FL</t>
         </is>
       </c>
       <c r="AA8" t="n">
@@ -1296,49 +1106,49 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46107</v>
+        <v>46086</v>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Texas Children's Houston Open</t>
+          <t>Arnold Palmer Invitational presented by Mastercard</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9900000</v>
+        <v>20000000</v>
       </c>
       <c r="E9" t="n">
-        <v>1782000</v>
+        <v>4000000</v>
       </c>
       <c r="F9" t="n">
-        <v>9900000</v>
+        <v>20000000</v>
       </c>
       <c r="G9" t="n">
-        <v>1782000</v>
+        <v>4000000</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Memorial Park</t>
+          <t>Bay Hill</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>897</v>
+        <v>9</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Min Woo Lee</t>
+          <t>Russel Henley</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r020?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r009?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1346,13 +1156,13 @@
         <v>72</v>
       </c>
       <c r="O9" t="n">
-        <v>7164</v>
+        <v>7381</v>
       </c>
       <c r="P9" t="n">
-        <v>73</v>
+        <v>75.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1371,91 +1181,95 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Orlando, FL</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Ernie Els</t>
         </is>
       </c>
       <c r="X9" t="n">
-        <v>-14</v>
+        <v>-16</v>
       </c>
       <c r="Y9" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>Memorial Park Golf Course, Houston TX</t>
+          <t>Bay Hill Club, Orlando FL</t>
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46114</v>
+        <v>46093</v>
       </c>
       <c r="B10" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Valero Texas Open</t>
+          <t>THE PLAYERS Championship</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>9800000</v>
+        <v>25000000</v>
       </c>
       <c r="E10" t="n">
-        <v>1764000</v>
+        <v>4500000</v>
       </c>
       <c r="F10" t="n">
-        <v>9800000</v>
+        <v>27777777.77</v>
       </c>
       <c r="G10" t="n">
-        <v>1764000</v>
+        <v>5000000</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TPC San Antonio</t>
+          <t>TPC Sawgrass</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>770</v>
+        <v>11</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Brian Harman</t>
+          <t>Rory McIlroy</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r041?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r011?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://www.theplayers.com/news/2026/03/09/media_1a0195f4b8db5ca190f4d05315255fc352cf9c37d.jpg?width=2000&amp;format=webply&amp;optimize=medium</t>
+        </is>
+      </c>
       <c r="N10" t="n">
         <v>72</v>
       </c>
       <c r="O10" t="n">
-        <v>7435</v>
+        <v>7245</v>
       </c>
       <c r="P10" t="n">
-        <v>75.40000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="Q10" t="n">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1474,7 +1288,7 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Ponte Vedra Beach, FL</t>
         </is>
       </c>
       <c r="V10" t="n">
@@ -1482,18 +1296,18 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Fred Couples / Greg Norman</t>
         </is>
       </c>
       <c r="X10" t="n">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="Y10" t="n">
         <v>-2</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>TPC San Antonio, San Antonio TX</t>
+          <t>TPC Sawgrass, Ponte Vedra Beach FL</t>
         </is>
       </c>
       <c r="AA10" t="n">
@@ -1502,67 +1316,63 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46121</v>
+        <v>46100</v>
       </c>
       <c r="B11" t="n">
-        <v>14</v>
+        <v>475</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Masters Tournament</t>
+          <t>Valspar Championship</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>21000000</v>
+        <v>9100000</v>
       </c>
       <c r="E11" t="n">
-        <v>4200000</v>
+        <v>1638000</v>
       </c>
       <c r="F11" t="n">
-        <v>27777777.77</v>
+        <v>9100000</v>
       </c>
       <c r="G11" t="n">
-        <v>5000000</v>
+        <v>1638000</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Augusta National</t>
+          <t>Innisbrook Resort</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>14</v>
+        <v>665</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>MAJOR</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Rory McIlroy</t>
+          <t>Viktor Hovland</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r014?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>https://photo-assets.masters.com/images/pics/tablet/m_25LW2_4788.jpg</t>
-        </is>
-      </c>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r475?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O11" t="n">
-        <v>7475</v>
+        <v>7340</v>
       </c>
       <c r="P11" t="n">
-        <v>78.09999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1581,7 +1391,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Augusta, GA</t>
+          <t>Palm Harbor, FL</t>
         </is>
       </c>
       <c r="V11" t="n">
@@ -1589,83 +1399,83 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Nick Price / Greg Norman</t>
+          <t>Multiple players</t>
         </is>
       </c>
       <c r="X11" t="n">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="Y11" t="n">
         <v>-1</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>Augusta National, Augusta GA</t>
+          <t>Innisbrook Resort, Palm Harbor FL</t>
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46128</v>
+        <v>46107</v>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RBC Heritage</t>
+          <t>Texas Children's Houston Open</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>20000000</v>
+        <v>9900000</v>
       </c>
       <c r="E12" t="n">
-        <v>3600000</v>
+        <v>1782000</v>
       </c>
       <c r="F12" t="n">
-        <v>20000000</v>
+        <v>9900000</v>
       </c>
       <c r="G12" t="n">
-        <v>3600000</v>
+        <v>1782000</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Harbour Town</t>
+          <t>Memorial Park</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>12</v>
+        <v>897</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Justin Thomas</t>
+          <t>Min Woo Lee</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r012?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r020?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O12" t="n">
-        <v>7099</v>
+        <v>7164</v>
       </c>
       <c r="P12" t="n">
-        <v>75.59999999999999</v>
+        <v>73</v>
       </c>
       <c r="Q12" t="n">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1684,73 +1494,77 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Hilton Head Island, SC</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Brian Gay</t>
+          <t>Multiple players</t>
         </is>
       </c>
       <c r="X12" t="n">
-        <v>-15</v>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>No Cut</t>
-        </is>
+        <v>-14</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>-2</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>Harbour Town Golf Links, Hilton Head SC</t>
-        </is>
-      </c>
-      <c r="AA12" t="inlineStr"/>
+          <t>Memorial Park Golf Course, Houston TX</t>
+        </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46142</v>
+        <v>46114</v>
       </c>
       <c r="B13" t="n">
-        <v>556</v>
+        <v>41</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cadillac Championship</t>
+          <t>Valero Texas Open</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>20000000</v>
+        <v>9800000</v>
       </c>
       <c r="E13" t="n">
-        <v>3600000</v>
+        <v>1764000</v>
       </c>
       <c r="F13" t="n">
-        <v>20000000</v>
+        <v>9800000</v>
       </c>
       <c r="G13" t="n">
-        <v>3600000</v>
+        <v>1764000</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Trump National Doral</t>
+          <t>TPC San Antonio</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>8</v>
+        <v>770</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Brian Harman</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r556?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r041?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1758,13 +1572,13 @@
         <v>72</v>
       </c>
       <c r="O13" t="n">
-        <v>7341</v>
+        <v>7435</v>
       </c>
       <c r="P13" t="n">
-        <v>75.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="Q13" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -1783,11 +1597,11 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -1795,83 +1609,87 @@
         </is>
       </c>
       <c r="X13" t="n">
-        <v>-19</v>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>No Cut</t>
-        </is>
+        <v>-13</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>-2</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>Trump National Doral, Miami FL</t>
-        </is>
-      </c>
-      <c r="AA13" t="inlineStr"/>
+          <t>TPC San Antonio, San Antonio TX</t>
+        </is>
+      </c>
+      <c r="AA13" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46149</v>
+        <v>46121</v>
       </c>
       <c r="B14" t="n">
-        <v>480</v>
+        <v>14</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Truist Championship</t>
+          <t>Masters Tournament</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>20000000</v>
+        <v>21000000</v>
       </c>
       <c r="E14" t="n">
-        <v>3600000</v>
+        <v>4200000</v>
       </c>
       <c r="F14" t="n">
-        <v>20000000</v>
+        <v>27777777.77</v>
       </c>
       <c r="G14" t="n">
-        <v>3600000</v>
+        <v>5000000</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Quail Hollow Club</t>
+          <t>Augusta National</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>872</v>
+        <v>14</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
+          <t>MAJOR</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Sepp Straka</t>
+          <t>Rory McIlroy</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r480?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r014?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://photo-assets.masters.com/images/pics/tablet/m_25LW2_4788.jpg</t>
+        </is>
+      </c>
       <c r="N14" t="n">
         <v>72</v>
       </c>
       <c r="O14" t="n">
-        <v>7635</v>
+        <v>7475</v>
       </c>
       <c r="P14" t="n">
-        <v>77.3</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1886,301 +1704,231 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Augusta, GA</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Rickie Fowler</t>
+          <t>Nick Price / Greg Norman</t>
         </is>
       </c>
       <c r="X14" t="n">
-        <v>-14</v>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>No Cut</t>
-        </is>
+        <v>-12</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>-1</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>Quail Hollow Club, Charlotte NC</t>
-        </is>
-      </c>
-      <c r="AA14" t="inlineStr"/>
+          <t>Augusta National, Augusta GA</t>
+        </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46156</v>
+        <v>46128</v>
       </c>
       <c r="B15" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PGA Championship</t>
+          <t>RBC Heritage</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>19000000</v>
+        <v>20000000</v>
       </c>
       <c r="E15" t="n">
-        <v>3420000</v>
+        <v>3600000</v>
       </c>
       <c r="F15" t="n">
-        <v>27777777.77</v>
+        <v>20000000</v>
       </c>
       <c r="G15" t="n">
-        <v>5000000</v>
+        <v>3600000</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Aronimink GC</t>
+          <t>Harbour Town</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>773</v>
+        <v>12</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>MAJOR</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Scottie Scheffler</t>
+          <t>Justin Thomas</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r033?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>https://pgachampionship.brightspotcdn.com/dims4/default/44f0a11/2147483647/strip/true/crop/6000x2917+0+542/resize/1920x933!/format/webp/quality/90/?url=http%3A%2F%2Fgolf-brightspot.s3.us-east-1.amazonaws.com%2Fpga%2F80%2F6b%2F2b2f0f4441a28b74ee8b18e21224%2Fagc-250602-151.jpg</t>
-        </is>
-      </c>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r012?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O15" t="n">
-        <v>7267</v>
+        <v>7099</v>
       </c>
       <c r="P15" t="n">
-        <v>75.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="Q15" t="n">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Ryegrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Newtown Square, PA</t>
+          <t>Hilton Head Island, SC</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Brian Gay</t>
         </is>
       </c>
       <c r="X15" t="n">
-        <v>-10</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>-1</v>
+        <v>-15</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>No Cut</t>
+        </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>Aronimink Golf Club, Newtown Square PA</t>
-        </is>
-      </c>
-      <c r="AA15" t="n">
-        <v>70</v>
-      </c>
+          <t>Harbour Town Golf Links, Hilton Head SC</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46163</v>
-      </c>
-      <c r="B16" t="n">
-        <v>19</v>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>THE CJ CUP Byron Nelson</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>10300000</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1854000</v>
-      </c>
-      <c r="F16" t="n">
-        <v>10300000</v>
-      </c>
+          <t>Miami Championship</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>1854000</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>TPC Craig Ranch</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>894</v>
-      </c>
+        <v>3600000</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Scottie Scheffler</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r019?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>72</v>
-      </c>
-      <c r="O16" t="n">
-        <v>7438</v>
-      </c>
-      <c r="P16" t="n">
-        <v>76.7</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>147</v>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Bentgrass</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Zoysia</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Bermuda</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>McKinney, TX</t>
-        </is>
-      </c>
-      <c r="V16" t="n">
-        <v>62</v>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>Multiple players</t>
-        </is>
-      </c>
-      <c r="X16" t="n">
-        <v>-21</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>-6</v>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>TPC Craig Ranch, McKinney TX</t>
-        </is>
-      </c>
-      <c r="AA16" t="n">
-        <v>65</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="B17" t="n">
-        <v>21</v>
+        <v>556</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Charles Schwab Challenge</t>
+          <t>Cadillac Championship</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>9900000</v>
+        <v>20000000</v>
       </c>
       <c r="E17" t="n">
-        <v>1782000</v>
+        <v>3600000</v>
       </c>
       <c r="F17" t="n">
-        <v>9900000</v>
+        <v>20000000</v>
       </c>
       <c r="G17" t="n">
-        <v>1782000</v>
+        <v>3600000</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Colonial Country Club</t>
+          <t>Trump National Doral</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Ben Griffin</t>
-        </is>
-      </c>
+          <t>SIGNATURE</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r023?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r556?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O17" t="n">
-        <v>7209</v>
+        <v>7341</v>
       </c>
       <c r="P17" t="n">
-        <v>74.5</v>
+        <v>75.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -2194,16 +1942,16 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Ryegrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Fort Worth, TX</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
@@ -2211,51 +1959,51 @@
         </is>
       </c>
       <c r="X17" t="n">
-        <v>-15</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>-3</v>
+        <v>-19</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>No Cut</t>
+        </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Colonial Country Club, Fort Worth TX</t>
-        </is>
-      </c>
-      <c r="AA17" t="n">
-        <v>65</v>
-      </c>
+          <t>Trump National Doral, Miami FL</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46177</v>
+        <v>46149</v>
       </c>
       <c r="B18" t="n">
-        <v>23</v>
+        <v>480</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>the Memorial Tournament presented by Workday</t>
+          <t>Truist Championship</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>20000000</v>
       </c>
       <c r="E18" t="n">
-        <v>4000000</v>
+        <v>3600000</v>
       </c>
       <c r="F18" t="n">
         <v>20000000</v>
       </c>
       <c r="G18" t="n">
-        <v>4000000</v>
+        <v>3600000</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Muirfield Village</t>
+          <t>Quail Hollow Club</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>23</v>
+        <v>872</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -2264,12 +2012,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Scottie Scheffler</t>
+          <t>Sepp Straka</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r032?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r480?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2277,13 +2025,13 @@
         <v>72</v>
       </c>
       <c r="O18" t="n">
-        <v>7392</v>
+        <v>7635</v>
       </c>
       <c r="P18" t="n">
-        <v>76.8</v>
+        <v>77.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -2292,17 +2040,17 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mix</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Dublin, OH</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="V18" t="n">
@@ -2310,83 +2058,87 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>Kenny Perry</t>
+          <t>Rickie Fowler</t>
         </is>
       </c>
       <c r="X18" t="n">
         <v>-14</v>
       </c>
-      <c r="Y18" t="n">
-        <v>-2</v>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>No Cut</t>
+        </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>Muirfield Village, Dublin OH</t>
-        </is>
-      </c>
-      <c r="AA18" t="n">
-        <v>50</v>
-      </c>
+          <t>Quail Hollow Club, Charlotte NC</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46184</v>
+        <v>46156</v>
       </c>
       <c r="B19" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>RBC Canadian Open</t>
+          <t>PGA Championship</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>9800000</v>
+        <v>19000000</v>
       </c>
       <c r="E19" t="n">
-        <v>1764000</v>
+        <v>3420000</v>
       </c>
       <c r="F19" t="n">
-        <v>9800000</v>
+        <v>27777777.77</v>
       </c>
       <c r="G19" t="n">
-        <v>1764000</v>
+        <v>5000000</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TPC Toronto</t>
+          <t>Aronimink GC</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>935</v>
+        <v>773</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>MAJOR</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Ryan Fox</t>
+          <t>Scottie Scheffler</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r032?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r033?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://pgachampionship.brightspotcdn.com/dims4/default/44f0a11/2147483647/strip/true/crop/6000x2917+0+542/resize/1920x933!/format/webp/quality/90/?url=http%3A%2F%2Fgolf-brightspot.s3.us-east-1.amazonaws.com%2Fpga%2F80%2F6b%2F2b2f0f4441a28b74ee8b18e21224%2Fagc-250602-151.jpg</t>
+        </is>
+      </c>
       <c r="N19" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="O19" t="n">
-        <v>7431</v>
+        <v>7267</v>
       </c>
       <c r="P19" t="n">
-        <v>76</v>
+        <v>75.5</v>
       </c>
       <c r="Q19" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -2395,21 +2147,21 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Zoysia</t>
+          <t>Bentgrass</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Mix</t>
+          <t>Ryegrass</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Oakville, ON, Canada</t>
+          <t>Newtown Square, PA</t>
         </is>
       </c>
       <c r="V19" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
@@ -2417,121 +2169,117 @@
         </is>
       </c>
       <c r="X19" t="n">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="Y19" t="n">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>TPC Toronto at Osprey Valley, Caledon Ontario</t>
+          <t>Aronimink Golf Club, Newtown Square PA</t>
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46191</v>
+        <v>46163</v>
       </c>
       <c r="B20" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>U.S. Open</t>
+          <t>THE CJ CUP Byron Nelson</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>21500000</v>
+        <v>10300000</v>
       </c>
       <c r="E20" t="n">
-        <v>4300000</v>
+        <v>1854000</v>
       </c>
       <c r="F20" t="n">
-        <v>27777777.77</v>
+        <v>10300000</v>
       </c>
       <c r="G20" t="n">
-        <v>5000000</v>
+        <v>1854000</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Shinnecock Hills GC</t>
+          <t>TPC Craig Ranch</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>618</v>
+        <v>894</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>MAJOR</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>J.J. Spaun</t>
+          <t>Scottie Scheffler</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r026?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>https://res.cloudinary.com/usga-single-app/image/upload/f_auto,fl_lossy,q_auto/c_fill,dpr_2.0,g_center/v1771360296/championships/usopen/images/2026/as-usopen-entries-open.jpg</t>
-        </is>
-      </c>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r019?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O20" t="n">
-        <v>7445</v>
+        <v>7438</v>
       </c>
       <c r="P20" t="n">
-        <v>74.5</v>
+        <v>76.7</v>
       </c>
       <c r="Q20" t="n">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Fescue</t>
+          <t>Bentgrass</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Fescue</t>
+          <t>Zoysia</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Fescue</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Southampton, NY</t>
+          <t>McKinney, TX</t>
         </is>
       </c>
       <c r="V20" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>Tommy Fleetwood</t>
+          <t>Multiple players</t>
         </is>
       </c>
       <c r="X20" t="n">
-        <v>-1</v>
+        <v>-21</v>
       </c>
       <c r="Y20" t="n">
-        <v>5</v>
+        <v>-6</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>Shinnecock Hills, Southampton NY</t>
+          <t>TPC Craig Ranch, McKinney TX</t>
         </is>
       </c>
       <c r="AA20" t="n">
@@ -2540,49 +2288,49 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46198</v>
+        <v>46170</v>
       </c>
       <c r="B21" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Travelers Championship</t>
+          <t>Charles Schwab Challenge</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>20000000</v>
+        <v>9900000</v>
       </c>
       <c r="E21" t="n">
-        <v>3600000</v>
+        <v>1782000</v>
       </c>
       <c r="F21" t="n">
-        <v>20000000</v>
+        <v>9900000</v>
       </c>
       <c r="G21" t="n">
-        <v>3600000</v>
+        <v>1782000</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TPC River Highlands</t>
+          <t>Colonial Country Club</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>503</v>
+        <v>21</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Keegan Bradley</t>
+          <t>Ben Griffin</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r034?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r023?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -2590,114 +2338,116 @@
         <v>70</v>
       </c>
       <c r="O21" t="n">
-        <v>6841</v>
+        <v>7209</v>
       </c>
       <c r="P21" t="n">
-        <v>73</v>
+        <v>74.5</v>
       </c>
       <c r="Q21" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mix</t>
+          <t>Ryegrass</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Cromwell, CT</t>
+          <t>Fort Worth, TX</t>
         </is>
       </c>
       <c r="V21" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>Jim Furyk</t>
+          <t>Multiple players</t>
         </is>
       </c>
       <c r="X21" t="n">
-        <v>-19</v>
+        <v>-15</v>
       </c>
       <c r="Y21" t="n">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>TPC River Highlands, Cromwell CT</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr"/>
+          <t>Colonial Country Club, Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46205</v>
+        <v>46177</v>
       </c>
       <c r="B22" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>John Deere Classic</t>
+          <t>the Memorial Tournament presented by Workday</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>8800000</v>
+        <v>20000000</v>
       </c>
       <c r="E22" t="n">
-        <v>1584000</v>
+        <v>4000000</v>
       </c>
       <c r="F22" t="n">
-        <v>8800000</v>
+        <v>20000000</v>
       </c>
       <c r="G22" t="n">
-        <v>1584000</v>
+        <v>4000000</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TPC Deere Run</t>
+          <t>Muirfield Village</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>669</v>
+        <v>23</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Brian Campbell</t>
+          <t>Scottie Scheffler</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r030?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r032?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O22" t="n">
-        <v>7281</v>
+        <v>7392</v>
       </c>
       <c r="P22" t="n">
-        <v>75.5</v>
+        <v>76.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -2716,63 +2466,63 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Silvis, IL</t>
+          <t>Dublin, OH</t>
         </is>
       </c>
       <c r="V22" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>Justin Thomas</t>
+          <t>Kenny Perry</t>
         </is>
       </c>
       <c r="X22" t="n">
-        <v>-20</v>
+        <v>-14</v>
       </c>
       <c r="Y22" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>TPC Deere Run, Silvis IL</t>
+          <t>Muirfield Village, Dublin OH</t>
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46212</v>
+        <v>46184</v>
       </c>
       <c r="B23" t="n">
-        <v>541</v>
+        <v>32</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Genesis Scottish Open</t>
+          <t>RBC Canadian Open</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9000000</v>
+        <v>9800000</v>
       </c>
       <c r="E23" t="n">
-        <v>1620000</v>
+        <v>1764000</v>
       </c>
       <c r="F23" t="n">
-        <v>9000000</v>
+        <v>9800000</v>
       </c>
       <c r="G23" t="n">
-        <v>1620000</v>
+        <v>1764000</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>The Renaissance Club</t>
+          <t>TPC Toronto</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>977</v>
+        <v>935</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -2781,45 +2531,45 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Chris Gotterup</t>
+          <t>Ryan Fox</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r541?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r032?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O23" t="n">
-        <v>7293</v>
+        <v>7431</v>
       </c>
       <c r="P23" t="n">
-        <v>73.5</v>
+        <v>76</v>
       </c>
       <c r="Q23" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Fescue</t>
+          <t>Bentgrass</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Fescue</t>
+          <t>Zoysia</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Fescue</t>
+          <t>Mix</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>North Berwick, Scotland</t>
+          <t>Oakville, ON, Canada</t>
         </is>
       </c>
       <c r="V23" t="n">
@@ -2831,14 +2581,14 @@
         </is>
       </c>
       <c r="X23" t="n">
-        <v>-17</v>
+        <v>-20</v>
       </c>
       <c r="Y23" t="n">
         <v>-5</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>The Renaissance Club, North Berwick Scotland</t>
+          <t>TPC Toronto at Osprey Valley, Caledon Ontario</t>
         </is>
       </c>
       <c r="AA23" t="n">
@@ -2847,21 +2597,21 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46219</v>
+        <v>46191</v>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>26</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Open Championship</t>
+          <t>U.S. Open</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>17000000</v>
+        <v>21500000</v>
       </c>
       <c r="E24" t="n">
-        <v>3100000</v>
+        <v>4300000</v>
       </c>
       <c r="F24" t="n">
         <v>27777777.77</v>
@@ -2871,11 +2621,11 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Royal Birkdale</t>
+          <t>Shinnecock Hills GC</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>541</v>
+        <v>618</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -2884,30 +2634,30 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Scottie Scheffler</t>
+          <t>J.J. Spaun</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r100?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r026?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://ichef.bbci.co.uk/ace/standard/1024/cpsprodpb/d72c/live/a1f81f10-4087-11ef-a3b9-c9442a06e32f.jpg</t>
+          <t>https://res.cloudinary.com/usga-single-app/image/upload/f_auto,fl_lossy,q_auto/c_fill,dpr_2.0,g_center/v1771360296/championships/usopen/images/2026/as-usopen-entries-open.jpg</t>
         </is>
       </c>
       <c r="N24" t="n">
         <v>70</v>
       </c>
       <c r="O24" t="n">
-        <v>7156</v>
+        <v>7445</v>
       </c>
       <c r="P24" t="n">
         <v>74.5</v>
       </c>
       <c r="Q24" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -2926,7 +2676,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Southport, England</t>
+          <t>Southampton, NY</t>
         </is>
       </c>
       <c r="V24" t="n">
@@ -2934,83 +2684,83 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>Mark Hayes</t>
+          <t>Tommy Fleetwood</t>
         </is>
       </c>
       <c r="X24" t="n">
-        <v>-12</v>
+        <v>-1</v>
       </c>
       <c r="Y24" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>Royal Birkdale, Southport England</t>
+          <t>Shinnecock Hills, Southampton NY</t>
         </is>
       </c>
       <c r="AA24" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46226</v>
+        <v>46198</v>
       </c>
       <c r="B25" t="n">
-        <v>525</v>
+        <v>34</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>3M Open</t>
+          <t>Travelers Championship</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8800000</v>
+        <v>20000000</v>
       </c>
       <c r="E25" t="n">
-        <v>1584000</v>
+        <v>3600000</v>
       </c>
       <c r="F25" t="n">
-        <v>8800000</v>
+        <v>20000000</v>
       </c>
       <c r="G25" t="n">
-        <v>1584000</v>
+        <v>3600000</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TPC Twin Cities</t>
+          <t>TPC River Highlands</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>883</v>
+        <v>503</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Kurt Kitayama</t>
+          <t>Keegan Bradley</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r525?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r034?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O25" t="n">
-        <v>7431</v>
+        <v>6841</v>
       </c>
       <c r="P25" t="n">
-        <v>75.5</v>
+        <v>73</v>
       </c>
       <c r="Q25" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -3024,68 +2774,66 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Ryegrass</t>
+          <t>Mix</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Blaine, MN</t>
+          <t>Cromwell, CT</t>
         </is>
       </c>
       <c r="V25" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>Matthew Wolff</t>
+          <t>Jim Furyk</t>
         </is>
       </c>
       <c r="X25" t="n">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="Y25" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>TPC Twin Cities, Blaine MN</t>
-        </is>
-      </c>
-      <c r="AA25" t="n">
-        <v>65</v>
-      </c>
+          <t>TPC River Highlands, Cromwell CT</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46233</v>
+        <v>46205</v>
       </c>
       <c r="B26" t="n">
-        <v>524</v>
+        <v>30</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Rocket Classic</t>
+          <t>John Deere Classic</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>10000000</v>
+        <v>8800000</v>
       </c>
       <c r="E26" t="n">
-        <v>1800000</v>
+        <v>1584000</v>
       </c>
       <c r="F26" t="n">
-        <v>10000000</v>
+        <v>8800000</v>
       </c>
       <c r="G26" t="n">
-        <v>1800000</v>
+        <v>1584000</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Detroit Golf Club</t>
+          <t>TPC Deere Run</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>876</v>
+        <v>669</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -3094,26 +2842,26 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Aldrich Potgieter</t>
+          <t>Brian Campbell</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r524?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r030?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O26" t="n">
-        <v>7341</v>
+        <v>7281</v>
       </c>
       <c r="P26" t="n">
-        <v>75</v>
+        <v>75.5</v>
       </c>
       <c r="Q26" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
@@ -3132,26 +2880,26 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Silvis, IL</t>
         </is>
       </c>
       <c r="V26" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Justin Thomas</t>
         </is>
       </c>
       <c r="X26" t="n">
-        <v>-23</v>
+        <v>-20</v>
       </c>
       <c r="Y26" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>Detroit Golf Club, Detroit MI</t>
+          <t>TPC Deere Run, Silvis IL</t>
         </is>
       </c>
       <c r="AA26" t="n">
@@ -3160,35 +2908,35 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46240</v>
+        <v>46212</v>
       </c>
       <c r="B27" t="n">
-        <v>13</v>
+        <v>541</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wyndham Championship</t>
+          <t>Genesis Scottish Open</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8500000</v>
+        <v>9000000</v>
       </c>
       <c r="E27" t="n">
-        <v>1530000</v>
+        <v>1620000</v>
       </c>
       <c r="F27" t="n">
-        <v>8500000</v>
+        <v>9000000</v>
       </c>
       <c r="G27" t="n">
-        <v>1530000</v>
+        <v>1620000</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Sedgefield Country Club</t>
+          <t>The Renaissance Club</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>752</v>
+        <v>977</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -3197,49 +2945,49 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Cameron Young</t>
+          <t>Chris Gotterup</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r013?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r541?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O27" t="n">
-        <v>7131</v>
+        <v>7293</v>
       </c>
       <c r="P27" t="n">
-        <v>74</v>
+        <v>73.5</v>
       </c>
       <c r="Q27" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Bentgrass</t>
+          <t>Fescue</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Fescue</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Fescue</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Greensboro, NC</t>
+          <t>North Berwick, Scotland</t>
         </is>
       </c>
       <c r="V27" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
@@ -3247,14 +2995,14 @@
         </is>
       </c>
       <c r="X27" t="n">
-        <v>-20</v>
+        <v>-17</v>
       </c>
       <c r="Y27" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>Sedgefield Country Club, Greensboro NC</t>
+          <t>The Renaissance Club, North Berwick Scotland</t>
         </is>
       </c>
       <c r="AA27" t="n">
@@ -3263,152 +3011,156 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46247</v>
+        <v>46219</v>
       </c>
       <c r="B28" t="n">
-        <v>27</v>
+        <v>100</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FedEx St. Jude Championship</t>
+          <t>The Open Championship</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>20000000</v>
+        <v>17000000</v>
       </c>
       <c r="E28" t="n">
-        <v>3600000</v>
+        <v>3100000</v>
       </c>
       <c r="F28" t="n">
-        <v>20000000</v>
+        <v>27777777.77</v>
       </c>
       <c r="G28" t="n">
-        <v>3600000</v>
+        <v>5000000</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>TPC Southwind</t>
+          <t>Royal Birkdale</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>513</v>
+        <v>541</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>PLAYOFFS</t>
+          <t>MAJOR</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Justin Rose</t>
+          <t>Scottie Scheffler</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r027?_a=DAJHqpB3ZAAB</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r100?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://ichef.bbci.co.uk/ace/standard/1024/cpsprodpb/d72c/live/a1f81f10-4087-11ef-a3b9-c9442a06e32f.jpg</t>
+        </is>
+      </c>
       <c r="N28" t="n">
         <v>70</v>
       </c>
       <c r="O28" t="n">
-        <v>7244</v>
+        <v>7156</v>
       </c>
       <c r="P28" t="n">
-        <v>74.59999999999999</v>
+        <v>74.5</v>
       </c>
       <c r="Q28" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Fescue</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Zoysia</t>
+          <t>Fescue</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Fescue</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Southport, England</t>
         </is>
       </c>
       <c r="V28" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Mark Hayes</t>
         </is>
       </c>
       <c r="X28" t="n">
-        <v>-17</v>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>No Cut</t>
-        </is>
+        <v>-12</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>-1</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>TPC Southwind, Memphis TN</t>
-        </is>
-      </c>
-      <c r="AA28" t="inlineStr"/>
+          <t>Royal Birkdale, Southport England</t>
+        </is>
+      </c>
+      <c r="AA28" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46254</v>
+        <v>46226</v>
       </c>
       <c r="B29" t="n">
-        <v>28</v>
+        <v>525</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BMW Championship</t>
+          <t>3M Open</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>20000000</v>
+        <v>8800000</v>
       </c>
       <c r="E29" t="n">
-        <v>3600000</v>
+        <v>1584000</v>
       </c>
       <c r="F29" t="n">
-        <v>20000000</v>
+        <v>8800000</v>
       </c>
       <c r="G29" t="n">
-        <v>3600000</v>
+        <v>1584000</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Bellerive CC</t>
+          <t>TPC Twin Cities</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>534</v>
+        <v>883</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>PLAYOFFS</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Scottie Scheffler</t>
+          <t>Kurt Kitayama</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r028?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r525?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -3416,13 +3168,13 @@
         <v>71</v>
       </c>
       <c r="O29" t="n">
-        <v>7547</v>
+        <v>7431</v>
       </c>
       <c r="P29" t="n">
-        <v>76.5</v>
+        <v>75.5</v>
       </c>
       <c r="Q29" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -3431,87 +3183,87 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Zoysia</t>
+          <t>Bentgrass</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Ryegrass</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Town and Country, MO</t>
+          <t>Blaine, MN</t>
         </is>
       </c>
       <c r="V29" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>Multiple players</t>
+          <t>Matthew Wolff</t>
         </is>
       </c>
       <c r="X29" t="n">
-        <v>-16</v>
-      </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>No Cut</t>
-        </is>
+        <v>-18</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>-5</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>Bellerive Country Club, St Louis MO</t>
-        </is>
-      </c>
-      <c r="AA29" t="inlineStr"/>
+          <t>TPC Twin Cities, Blaine MN</t>
+        </is>
+      </c>
+      <c r="AA29" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46261</v>
+        <v>46233</v>
       </c>
       <c r="B30" t="n">
-        <v>60</v>
+        <v>524</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tour Championship</t>
+          <t>Rocket Classic</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>40000000</v>
+        <v>10000000</v>
       </c>
       <c r="E30" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F30" t="n">
         <v>10000000</v>
       </c>
-      <c r="F30" t="n">
-        <v>27777777.77</v>
-      </c>
       <c r="G30" t="n">
-        <v>5000000</v>
+        <v>1800000</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>East Lake</t>
+          <t>Detroit Golf Club</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>933</v>
+        <v>876</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>PLAYOFFS</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Tommy Fleetwood</t>
+          <t>Aldrich Potgieter</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r060?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r524?_a=DAJHqpB3ZAAB</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -3519,7 +3271,7 @@
         <v>72</v>
       </c>
       <c r="O30" t="n">
-        <v>7346</v>
+        <v>7341</v>
       </c>
       <c r="P30" t="n">
         <v>75</v>
@@ -3529,22 +3281,22 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Bentgrass</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Bentgrass</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Mix</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="V30" t="n">
@@ -3556,19 +3308,431 @@
         </is>
       </c>
       <c r="X30" t="n">
+        <v>-23</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>-7</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>Detroit Golf Club, Detroit MI</t>
+        </is>
+      </c>
+      <c r="AA30" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B31" t="n">
+        <v>13</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Wyndham Championship</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1530000</v>
+      </c>
+      <c r="F31" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1530000</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Sedgefield Country Club</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>752</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Cameron Young</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r013?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="n">
+        <v>70</v>
+      </c>
+      <c r="O31" t="n">
+        <v>7131</v>
+      </c>
+      <c r="P31" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>130</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Bentgrass</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Greensboro, NC</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>60</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Multiple players</t>
+        </is>
+      </c>
+      <c r="X31" t="n">
+        <v>-20</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>-6</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>Sedgefield Country Club, Greensboro NC</t>
+        </is>
+      </c>
+      <c r="AA31" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B32" t="n">
+        <v>27</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>FedEx St. Jude Championship</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="F32" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>TPC Southwind</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>513</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>PLAYOFFS</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Justin Rose</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r027?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>70</v>
+      </c>
+      <c r="O32" t="n">
+        <v>7244</v>
+      </c>
+      <c r="P32" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>136</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Zoysia</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Memphis, TN</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>61</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Multiple players</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
+        <v>-17</v>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>No Cut</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>TPC Southwind, Memphis TN</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B33" t="n">
+        <v>28</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BMW Championship</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="F33" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="G33" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Bellerive CC</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>534</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>PLAYOFFS</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Scottie Scheffler</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r028?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="n">
+        <v>71</v>
+      </c>
+      <c r="O33" t="n">
+        <v>7547</v>
+      </c>
+      <c r="P33" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>141</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Bentgrass</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Zoysia</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Town and Country, MO</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>62</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Multiple players</t>
+        </is>
+      </c>
+      <c r="X33" t="n">
+        <v>-16</v>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>No Cut</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Bellerive Country Club, St Louis MO</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B34" t="n">
+        <v>60</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Tour Championship</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="E34" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="F34" t="n">
+        <v>27777777.77</v>
+      </c>
+      <c r="G34" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>East Lake</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>933</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>PLAYOFFS</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Tommy Fleetwood</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r060?_a=DAJHqpB3ZAAB</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="n">
+        <v>72</v>
+      </c>
+      <c r="O34" t="n">
+        <v>7346</v>
+      </c>
+      <c r="P34" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>135</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>61</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Multiple players</t>
+        </is>
+      </c>
+      <c r="X34" t="n">
         <v>-14</v>
       </c>
-      <c r="Y30" t="inlineStr">
+      <c r="Y34" t="inlineStr">
         <is>
           <t>No Cut</t>
         </is>
       </c>
-      <c r="Z30" t="inlineStr">
+      <c r="Z34" t="inlineStr">
         <is>
           <t>East Lake Golf Club, Atlanta GA</t>
         </is>
       </c>
-      <c r="AA30" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: OAD 3.5k field/odds gating, ownership math, overview panel sizing
- Fix odds disabled for next-week events (matched_from_this_week flag)
- Derive our_used from events CSVs instead of stale JSON
- Fix event selector stable key to preserve user selection
- Fix overview favourites/hottest panels to render in single st.markdown call
- Add truist_championship.csv and fix miami_championship.csv dg_ids
- Update OAD_2026_Schedule.xlsx purse/winner_share values

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/in Use/OAD_2026_Schedule.xlsx
+++ b/Data/in Use/OAD_2026_Schedule.xlsx
@@ -579,11 +579,17 @@
           <t>Sony Open in Hawaii</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>9100000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1638000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>9100000</v>
+      </c>
       <c r="G2" t="n">
-        <v>991900</v>
+        <v>1638000</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -620,11 +626,17 @@
           <t>The American Express</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>9200000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1656000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9200000</v>
+      </c>
       <c r="G3" t="n">
-        <v>616400</v>
+        <v>1656000</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -2089,10 +2101,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>19000000</v>
+        <v>20000000</v>
       </c>
       <c r="E19" t="n">
-        <v>3420000</v>
+        <v>3600000</v>
       </c>
       <c r="F19" t="n">
         <v>27777777.77</v>

</xml_diff>

<commit_message>
fix: CJ Cup odds gating, course history, OAD leaderboard, overview sizing
- Block stale PGA odds from showing on CJ Cup (event_name mismatch check)
- Normalize TPC Craig Ranch course_num 894→921 across all data files
- Add _COURSE_NUM_EQUIV for same-venue course num aliases in overview
- Add CJ Cup banner image URL to schedule
- OAD 3.5k: our_used derived from events CSVs, ahead/behind % fix
- Overview favourites/hottest panels rendered in single st.markdown call
- Add pga_championship.csv OAD event (auto-applies to 3.5k leaderboard)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/in Use/OAD_2026_Schedule.xlsx
+++ b/Data/in Use/OAD_2026_Schedule.xlsx
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>894</v>
+        <v>921</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/pgatour-prod/image/upload/dpr_2.0,q_auto/c_scale,w_200/v1/tournaments/logos/r019?_a=DAJHqpB3ZAAB</t>
+          <t>https://res.cloudinary.com/pgatour-prod/d_tournaments:logos:R000.png/tournaments/logos/R019.png</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>

</xml_diff>